<commit_message>
Implement Supabase real-time dual-sync integration and render connectivity status indicator badge in dashboard header
</commit_message>
<xml_diff>
--- a/tests/reports/appium_test_report.xlsx
+++ b/tests/reports/appium_test_report.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="J3" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="J9" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="J13" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="J15" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="J19" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="J21" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="J23" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="J27" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="J29" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="J31" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="J33" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="J34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="J35" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="J37" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="J39" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="J41" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="J43" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3763,7 @@
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="J45" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="J47" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="J49" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="J53" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="J55" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="J57" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
       </c>
       <c r="J58" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="J59" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="J61" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="J63" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="J65" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="J66" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="J67" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="J68" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="J69" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="J70" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="J71" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="J72" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="J73" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J74" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="J75" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="J76" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="J77" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="J78" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5591,7 +5591,7 @@
       </c>
       <c r="J79" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="J80" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="J81" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
       </c>
       <c r="J82" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="J83" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5855,7 +5855,7 @@
       </c>
       <c r="J84" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="J85" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="J86" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6013,7 +6013,7 @@
       </c>
       <c r="J87" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="J88" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6117,7 @@
       </c>
       <c r="J89" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="J90" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="J91" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="J92" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6326,7 +6326,7 @@
       </c>
       <c r="J93" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="J94" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="J95" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="J96" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="J97" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6592,7 +6592,7 @@
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6644,7 @@
       </c>
       <c r="J99" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="J101" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J102" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="J103" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="J104" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="J105" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7011,7 @@
       </c>
       <c r="J106" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="J107" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7116,7 +7116,7 @@
       </c>
       <c r="J108" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7168,7 +7168,7 @@
       </c>
       <c r="J109" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7220,7 @@
       </c>
       <c r="J110" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7273,7 +7273,7 @@
       </c>
       <c r="J111" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="J112" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="J113" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="J114" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="J115" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="J116" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       </c>
       <c r="J117" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7638,7 +7638,7 @@
       </c>
       <c r="J118" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7691,7 @@
       </c>
       <c r="J119" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="J120" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7796,7 +7796,7 @@
       </c>
       <c r="J121" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="J122" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="J123" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -7955,7 +7955,7 @@
       </c>
       <c r="J124" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="J125" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8061,7 +8061,7 @@
       </c>
       <c r="J126" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="J127" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8167,7 +8167,7 @@
       </c>
       <c r="J128" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="J129" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="J130" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8323,7 +8323,7 @@
       </c>
       <c r="J131" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="J132" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8427,7 +8427,7 @@
       </c>
       <c r="J133" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="J134" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8531,7 +8531,7 @@
       </c>
       <c r="J135" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="J136" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8636,7 +8636,7 @@
       </c>
       <c r="J137" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8688,7 +8688,7 @@
       </c>
       <c r="J138" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="J139" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8792,7 +8792,7 @@
       </c>
       <c r="J140" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8845,7 +8845,7 @@
       </c>
       <c r="J141" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="J142" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J143" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9003,7 +9003,7 @@
       </c>
       <c r="J144" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="J145" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="J146" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9160,7 @@
       </c>
       <c r="J147" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9212,7 @@
       </c>
       <c r="J148" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9264,7 @@
       </c>
       <c r="J149" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="J150" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="J151" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9421,7 @@
       </c>
       <c r="J152" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="J153" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="J154" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="J155" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9633,7 +9633,7 @@
       </c>
       <c r="J156" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9686,7 +9686,7 @@
       </c>
       <c r="J157" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9739,7 @@
       </c>
       <c r="J158" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9791,7 +9791,7 @@
       </c>
       <c r="J159" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9844,7 +9844,7 @@
       </c>
       <c r="J160" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9897,7 +9897,7 @@
       </c>
       <c r="J161" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -9949,7 +9949,7 @@
       </c>
       <c r="J162" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="J163" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="J164" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="J165" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10159,7 +10159,7 @@
       </c>
       <c r="J166" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10211,7 +10211,7 @@
       </c>
       <c r="J167" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="J168" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10316,7 +10316,7 @@
       </c>
       <c r="J169" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="J170" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="J171" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10473,7 +10473,7 @@
       </c>
       <c r="J172" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10525,7 +10525,7 @@
       </c>
       <c r="J173" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10577,7 +10577,7 @@
       </c>
       <c r="J174" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="J175" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10681,7 +10681,7 @@
       </c>
       <c r="J176" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10733,7 +10733,7 @@
       </c>
       <c r="J177" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10785,7 +10785,7 @@
       </c>
       <c r="J178" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10837,7 +10837,7 @@
       </c>
       <c r="J179" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="J180" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="J181" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -10994,7 +10994,7 @@
       </c>
       <c r="J182" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11046,7 +11046,7 @@
       </c>
       <c r="J183" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11098,7 +11098,7 @@
       </c>
       <c r="J184" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11150,7 +11150,7 @@
       </c>
       <c r="J185" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11203,7 +11203,7 @@
       </c>
       <c r="J186" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11255,7 +11255,7 @@
       </c>
       <c r="J187" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="J188" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11359,7 +11359,7 @@
       </c>
       <c r="J189" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11411,7 +11411,7 @@
       </c>
       <c r="J190" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="J191" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11515,7 @@
       </c>
       <c r="J192" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11567,7 +11567,7 @@
       </c>
       <c r="J193" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11619,7 +11619,7 @@
       </c>
       <c r="J194" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11671,7 +11671,7 @@
       </c>
       <c r="J195" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="J196" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11775,7 +11775,7 @@
       </c>
       <c r="J197" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11827,7 +11827,7 @@
       </c>
       <c r="J198" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="J199" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11932,7 +11932,7 @@
       </c>
       <c r="J200" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -11984,7 +11984,7 @@
       </c>
       <c r="J201" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12036,7 +12036,7 @@
       </c>
       <c r="J202" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12088,7 +12088,7 @@
       </c>
       <c r="J203" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="J204" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12192,7 +12192,7 @@
       </c>
       <c r="J205" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12244,7 +12244,7 @@
       </c>
       <c r="J206" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12296,7 +12296,7 @@
       </c>
       <c r="J207" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="J208" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="J209" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12452,7 +12452,7 @@
       </c>
       <c r="J210" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12504,7 +12504,7 @@
       </c>
       <c r="J211" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12556,7 +12556,7 @@
       </c>
       <c r="J212" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12608,7 +12608,7 @@
       </c>
       <c r="J213" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12660,7 @@
       </c>
       <c r="J214" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12712,7 +12712,7 @@
       </c>
       <c r="J215" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12764,7 +12764,7 @@
       </c>
       <c r="J216" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12816,7 +12816,7 @@
       </c>
       <c r="J217" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12868,7 +12868,7 @@
       </c>
       <c r="J218" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="J219" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -12973,7 +12973,7 @@
       </c>
       <c r="J220" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13025,7 +13025,7 @@
       </c>
       <c r="J221" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13077,7 +13077,7 @@
       </c>
       <c r="J222" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13129,7 +13129,7 @@
       </c>
       <c r="J223" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13181,7 +13181,7 @@
       </c>
       <c r="J224" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13233,7 +13233,7 @@
       </c>
       <c r="J225" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13285,7 +13285,7 @@
       </c>
       <c r="J226" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13337,7 +13337,7 @@
       </c>
       <c r="J227" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13389,7 +13389,7 @@
       </c>
       <c r="J228" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="J229" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13493,7 +13493,7 @@
       </c>
       <c r="J230" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13545,7 +13545,7 @@
       </c>
       <c r="J231" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13597,7 +13597,7 @@
       </c>
       <c r="J232" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13649,7 @@
       </c>
       <c r="J233" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13701,7 +13701,7 @@
       </c>
       <c r="J234" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13753,7 +13753,7 @@
       </c>
       <c r="J235" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13805,7 +13805,7 @@
       </c>
       <c r="J236" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13857,7 +13857,7 @@
       </c>
       <c r="J237" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13909,7 +13909,7 @@
       </c>
       <c r="J238" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -13961,7 +13961,7 @@
       </c>
       <c r="J239" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14013,7 +14013,7 @@
       </c>
       <c r="J240" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14065,7 +14065,7 @@
       </c>
       <c r="J241" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14118,7 +14118,7 @@
       </c>
       <c r="J242" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14170,7 +14170,7 @@
       </c>
       <c r="J243" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14222,7 +14222,7 @@
       </c>
       <c r="J244" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14274,7 +14274,7 @@
       </c>
       <c r="J245" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14327,7 +14327,7 @@
       </c>
       <c r="J246" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14380,7 +14380,7 @@
       </c>
       <c r="J247" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14432,7 +14432,7 @@
       </c>
       <c r="J248" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14484,7 +14484,7 @@
       </c>
       <c r="J249" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14536,7 +14536,7 @@
       </c>
       <c r="J250" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14589,7 +14589,7 @@
       </c>
       <c r="J251" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14641,7 +14641,7 @@
       </c>
       <c r="J252" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14693,7 +14693,7 @@
       </c>
       <c r="J253" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="J254" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14797,7 +14797,7 @@
       </c>
       <c r="J255" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14850,7 +14850,7 @@
       </c>
       <c r="J256" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14902,7 +14902,7 @@
       </c>
       <c r="J257" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -14954,7 +14954,7 @@
       </c>
       <c r="J258" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15006,7 +15006,7 @@
       </c>
       <c r="J259" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15058,7 +15058,7 @@
       </c>
       <c r="J260" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15110,7 +15110,7 @@
       </c>
       <c r="J261" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15162,7 +15162,7 @@
       </c>
       <c r="J262" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15214,7 +15214,7 @@
       </c>
       <c r="J263" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15267,7 +15267,7 @@
       </c>
       <c r="J264" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15319,7 +15319,7 @@
       </c>
       <c r="J265" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15371,7 +15371,7 @@
       </c>
       <c r="J266" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15423,7 +15423,7 @@
       </c>
       <c r="J267" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15475,7 +15475,7 @@
       </c>
       <c r="J268" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15527,7 +15527,7 @@
       </c>
       <c r="J269" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15579,7 +15579,7 @@
       </c>
       <c r="J270" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15631,7 +15631,7 @@
       </c>
       <c r="J271" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15683,7 +15683,7 @@
       </c>
       <c r="J272" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15735,7 +15735,7 @@
       </c>
       <c r="J273" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15787,7 +15787,7 @@
       </c>
       <c r="J274" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15839,7 +15839,7 @@
       </c>
       <c r="J275" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15891,7 +15891,7 @@
       </c>
       <c r="J276" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15943,7 +15943,7 @@
       </c>
       <c r="J277" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -15996,7 +15996,7 @@
       </c>
       <c r="J278" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16048,7 +16048,7 @@
       </c>
       <c r="J279" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16100,7 +16100,7 @@
       </c>
       <c r="J280" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16153,7 +16153,7 @@
       </c>
       <c r="J281" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16205,7 +16205,7 @@
       </c>
       <c r="J282" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16257,7 +16257,7 @@
       </c>
       <c r="J283" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16309,7 +16309,7 @@
       </c>
       <c r="J284" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="J285" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16413,7 +16413,7 @@
       </c>
       <c r="J286" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16465,7 +16465,7 @@
       </c>
       <c r="J287" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16517,7 +16517,7 @@
       </c>
       <c r="J288" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16569,7 +16569,7 @@
       </c>
       <c r="J289" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16622,7 +16622,7 @@
       </c>
       <c r="J290" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16675,7 +16675,7 @@
       </c>
       <c r="J291" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16727,7 +16727,7 @@
       </c>
       <c r="J292" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16779,7 +16779,7 @@
       </c>
       <c r="J293" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16831,7 +16831,7 @@
       </c>
       <c r="J294" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16883,7 +16883,7 @@
       </c>
       <c r="J295" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16935,7 +16935,7 @@
       </c>
       <c r="J296" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -16987,7 +16987,7 @@
       </c>
       <c r="J297" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -17039,7 +17039,7 @@
       </c>
       <c r="J298" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="J299" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -17144,7 +17144,7 @@
       </c>
       <c r="J300" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>
@@ -17196,7 +17196,7 @@
       </c>
       <c r="J301" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 19:57:37</t>
+          <t>2026-07-23 20:08:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Excel export, community live polling+replies, dark theme, wellness spinner
</commit_message>
<xml_diff>
--- a/tests/reports/appium_test_report.xlsx
+++ b/tests/reports/appium_test_report.xlsx
@@ -584,7 +584,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="J2" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="J3" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1723,7 +1723,7 @@
       </c>
       <c r="J5" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1775,7 @@
       </c>
       <c r="J6" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="J7" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="J8" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="J9" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="J10" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2038,7 @@
       </c>
       <c r="J11" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2091,7 @@
       </c>
       <c r="J12" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2144,7 @@
       </c>
       <c r="J13" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="J14" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="J15" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2303,7 +2303,7 @@
       </c>
       <c r="J16" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="J17" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="J18" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2461,7 +2461,7 @@
       </c>
       <c r="J19" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="J20" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
       </c>
       <c r="J21" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="J22" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="J23" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="J25" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
       </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="J27" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J28" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2981,7 @@
       </c>
       <c r="J29" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3033,7 +3033,7 @@
       </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3086,7 @@
       </c>
       <c r="J31" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="J32" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="J33" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="J34" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="J35" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="J36" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="J37" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="J38" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="J39" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="J40" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="J41" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="J42" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="J43" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3763,7 @@
       </c>
       <c r="J44" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="J45" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="J46" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="J47" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -3971,7 +3971,7 @@
       </c>
       <c r="J48" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="J49" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4075,7 +4075,7 @@
       </c>
       <c r="J50" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="J51" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="J52" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
       </c>
       <c r="J53" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
       </c>
       <c r="J54" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4336,7 @@
       </c>
       <c r="J55" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4388,7 +4388,7 @@
       </c>
       <c r="J56" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="J57" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
       </c>
       <c r="J58" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4545,7 @@
       </c>
       <c r="J59" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J60" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="J61" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="J62" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4755,7 +4755,7 @@
       </c>
       <c r="J63" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="J64" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="J65" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="J66" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="J67" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="J68" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="J69" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="J70" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5173,7 +5173,7 @@
       </c>
       <c r="J71" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="J72" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="J73" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J74" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5381,7 +5381,7 @@
       </c>
       <c r="J75" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5433,7 @@
       </c>
       <c r="J76" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="J77" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5538,7 +5538,7 @@
       </c>
       <c r="J78" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5591,7 +5591,7 @@
       </c>
       <c r="J79" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5643,7 +5643,7 @@
       </c>
       <c r="J80" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5695,7 @@
       </c>
       <c r="J81" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5749,7 +5749,7 @@
       </c>
       <c r="J82" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="J83" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5855,7 +5855,7 @@
       </c>
       <c r="J84" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="J85" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="J86" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6013,7 +6013,7 @@
       </c>
       <c r="J87" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="J88" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6117,7 +6117,7 @@
       </c>
       <c r="J89" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6169,7 +6169,7 @@
       </c>
       <c r="J90" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6221,7 @@
       </c>
       <c r="J91" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6274,7 +6274,7 @@
       </c>
       <c r="J92" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6326,7 +6326,7 @@
       </c>
       <c r="J93" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="J94" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6432,7 +6432,7 @@
       </c>
       <c r="J95" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="J96" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6540,7 +6540,7 @@
       </c>
       <c r="J97" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6592,7 +6592,7 @@
       </c>
       <c r="J98" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6644,7 @@
       </c>
       <c r="J99" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6696,7 +6696,7 @@
       </c>
       <c r="J100" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
       </c>
       <c r="J101" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J102" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6852,7 +6852,7 @@
       </c>
       <c r="J103" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6905,7 +6905,7 @@
       </c>
       <c r="J104" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -6958,7 +6958,7 @@
       </c>
       <c r="J105" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7011,7 +7011,7 @@
       </c>
       <c r="J106" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="J107" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7116,7 +7116,7 @@
       </c>
       <c r="J108" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7168,7 +7168,7 @@
       </c>
       <c r="J109" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7220,7 +7220,7 @@
       </c>
       <c r="J110" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7273,7 +7273,7 @@
       </c>
       <c r="J111" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="J112" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
       </c>
       <c r="J113" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="J114" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7481,7 +7481,7 @@
       </c>
       <c r="J115" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7533,7 +7533,7 @@
       </c>
       <c r="J116" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
       </c>
       <c r="J117" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7638,7 +7638,7 @@
       </c>
       <c r="J118" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7691,7 @@
       </c>
       <c r="J119" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="J120" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7796,7 +7796,7 @@
       </c>
       <c r="J121" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7849,7 +7849,7 @@
       </c>
       <c r="J122" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7902,7 @@
       </c>
       <c r="J123" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -7955,7 +7955,7 @@
       </c>
       <c r="J124" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="J125" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8061,7 +8061,7 @@
       </c>
       <c r="J126" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="J127" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8167,7 +8167,7 @@
       </c>
       <c r="J128" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="J129" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
       </c>
       <c r="J130" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8323,7 +8323,7 @@
       </c>
       <c r="J131" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="J132" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8427,7 +8427,7 @@
       </c>
       <c r="J133" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="J134" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8531,7 +8531,7 @@
       </c>
       <c r="J135" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8584,7 +8584,7 @@
       </c>
       <c r="J136" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8636,7 +8636,7 @@
       </c>
       <c r="J137" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8688,7 +8688,7 @@
       </c>
       <c r="J138" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="J139" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8792,7 +8792,7 @@
       </c>
       <c r="J140" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8845,7 +8845,7 @@
       </c>
       <c r="J141" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="J142" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -8950,7 +8950,7 @@
       </c>
       <c r="J143" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9003,7 +9003,7 @@
       </c>
       <c r="J144" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="J145" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="J146" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9160,7 @@
       </c>
       <c r="J147" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9212,7 +9212,7 @@
       </c>
       <c r="J148" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9264,7 @@
       </c>
       <c r="J149" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9316,7 +9316,7 @@
       </c>
       <c r="J150" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="J151" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9421,7 +9421,7 @@
       </c>
       <c r="J152" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="J153" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9526,7 +9526,7 @@
       </c>
       <c r="J154" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="J155" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9633,7 +9633,7 @@
       </c>
       <c r="J156" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9686,7 +9686,7 @@
       </c>
       <c r="J157" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9739,7 @@
       </c>
       <c r="J158" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9791,7 +9791,7 @@
       </c>
       <c r="J159" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9844,7 +9844,7 @@
       </c>
       <c r="J160" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9897,7 +9897,7 @@
       </c>
       <c r="J161" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -9949,7 +9949,7 @@
       </c>
       <c r="J162" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10001,7 +10001,7 @@
       </c>
       <c r="J163" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10054,7 +10054,7 @@
       </c>
       <c r="J164" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10106,7 +10106,7 @@
       </c>
       <c r="J165" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10159,7 +10159,7 @@
       </c>
       <c r="J166" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10211,7 +10211,7 @@
       </c>
       <c r="J167" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10263,7 +10263,7 @@
       </c>
       <c r="J168" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10316,7 +10316,7 @@
       </c>
       <c r="J169" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10368,7 +10368,7 @@
       </c>
       <c r="J170" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10420,7 +10420,7 @@
       </c>
       <c r="J171" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10473,7 +10473,7 @@
       </c>
       <c r="J172" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10525,7 +10525,7 @@
       </c>
       <c r="J173" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10577,7 +10577,7 @@
       </c>
       <c r="J174" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="J175" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10681,7 +10681,7 @@
       </c>
       <c r="J176" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10733,7 +10733,7 @@
       </c>
       <c r="J177" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10785,7 +10785,7 @@
       </c>
       <c r="J178" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10837,7 +10837,7 @@
       </c>
       <c r="J179" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="J180" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="J181" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -10994,7 +10994,7 @@
       </c>
       <c r="J182" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11046,7 +11046,7 @@
       </c>
       <c r="J183" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11098,7 +11098,7 @@
       </c>
       <c r="J184" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11150,7 +11150,7 @@
       </c>
       <c r="J185" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11203,7 +11203,7 @@
       </c>
       <c r="J186" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11255,7 +11255,7 @@
       </c>
       <c r="J187" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11307,7 +11307,7 @@
       </c>
       <c r="J188" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11359,7 +11359,7 @@
       </c>
       <c r="J189" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11411,7 +11411,7 @@
       </c>
       <c r="J190" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11463,7 +11463,7 @@
       </c>
       <c r="J191" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11515,7 @@
       </c>
       <c r="J192" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11567,7 +11567,7 @@
       </c>
       <c r="J193" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11619,7 +11619,7 @@
       </c>
       <c r="J194" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11671,7 +11671,7 @@
       </c>
       <c r="J195" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="J196" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11775,7 +11775,7 @@
       </c>
       <c r="J197" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11827,7 +11827,7 @@
       </c>
       <c r="J198" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="J199" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11932,7 +11932,7 @@
       </c>
       <c r="J200" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -11984,7 +11984,7 @@
       </c>
       <c r="J201" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12036,7 +12036,7 @@
       </c>
       <c r="J202" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12088,7 +12088,7 @@
       </c>
       <c r="J203" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12140,7 +12140,7 @@
       </c>
       <c r="J204" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12192,7 +12192,7 @@
       </c>
       <c r="J205" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12244,7 +12244,7 @@
       </c>
       <c r="J206" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12296,7 +12296,7 @@
       </c>
       <c r="J207" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="J208" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="J209" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12452,7 +12452,7 @@
       </c>
       <c r="J210" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12504,7 +12504,7 @@
       </c>
       <c r="J211" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12556,7 +12556,7 @@
       </c>
       <c r="J212" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12608,7 +12608,7 @@
       </c>
       <c r="J213" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12660,7 +12660,7 @@
       </c>
       <c r="J214" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12712,7 +12712,7 @@
       </c>
       <c r="J215" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12764,7 +12764,7 @@
       </c>
       <c r="J216" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12816,7 +12816,7 @@
       </c>
       <c r="J217" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12868,7 +12868,7 @@
       </c>
       <c r="J218" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12921,7 +12921,7 @@
       </c>
       <c r="J219" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -12973,7 +12973,7 @@
       </c>
       <c r="J220" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13025,7 +13025,7 @@
       </c>
       <c r="J221" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13077,7 +13077,7 @@
       </c>
       <c r="J222" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13129,7 +13129,7 @@
       </c>
       <c r="J223" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13181,7 +13181,7 @@
       </c>
       <c r="J224" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13233,7 +13233,7 @@
       </c>
       <c r="J225" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13285,7 +13285,7 @@
       </c>
       <c r="J226" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13337,7 +13337,7 @@
       </c>
       <c r="J227" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13389,7 +13389,7 @@
       </c>
       <c r="J228" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13441,7 +13441,7 @@
       </c>
       <c r="J229" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13493,7 +13493,7 @@
       </c>
       <c r="J230" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13545,7 +13545,7 @@
       </c>
       <c r="J231" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13597,7 +13597,7 @@
       </c>
       <c r="J232" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13649,7 +13649,7 @@
       </c>
       <c r="J233" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13701,7 +13701,7 @@
       </c>
       <c r="J234" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13753,7 +13753,7 @@
       </c>
       <c r="J235" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13805,7 +13805,7 @@
       </c>
       <c r="J236" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13857,7 +13857,7 @@
       </c>
       <c r="J237" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13909,7 +13909,7 @@
       </c>
       <c r="J238" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -13961,7 +13961,7 @@
       </c>
       <c r="J239" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14013,7 +14013,7 @@
       </c>
       <c r="J240" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14065,7 +14065,7 @@
       </c>
       <c r="J241" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14118,7 +14118,7 @@
       </c>
       <c r="J242" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14170,7 +14170,7 @@
       </c>
       <c r="J243" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14222,7 +14222,7 @@
       </c>
       <c r="J244" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14274,7 +14274,7 @@
       </c>
       <c r="J245" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14327,7 +14327,7 @@
       </c>
       <c r="J246" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14380,7 +14380,7 @@
       </c>
       <c r="J247" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14432,7 +14432,7 @@
       </c>
       <c r="J248" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14484,7 +14484,7 @@
       </c>
       <c r="J249" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14536,7 +14536,7 @@
       </c>
       <c r="J250" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14589,7 +14589,7 @@
       </c>
       <c r="J251" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14641,7 +14641,7 @@
       </c>
       <c r="J252" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14693,7 +14693,7 @@
       </c>
       <c r="J253" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="J254" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14797,7 +14797,7 @@
       </c>
       <c r="J255" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14850,7 +14850,7 @@
       </c>
       <c r="J256" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14902,7 +14902,7 @@
       </c>
       <c r="J257" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -14954,7 +14954,7 @@
       </c>
       <c r="J258" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15006,7 +15006,7 @@
       </c>
       <c r="J259" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15058,7 +15058,7 @@
       </c>
       <c r="J260" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15110,7 +15110,7 @@
       </c>
       <c r="J261" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15162,7 +15162,7 @@
       </c>
       <c r="J262" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15214,7 +15214,7 @@
       </c>
       <c r="J263" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15267,7 +15267,7 @@
       </c>
       <c r="J264" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15319,7 +15319,7 @@
       </c>
       <c r="J265" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15371,7 +15371,7 @@
       </c>
       <c r="J266" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15423,7 +15423,7 @@
       </c>
       <c r="J267" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15475,7 +15475,7 @@
       </c>
       <c r="J268" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15527,7 +15527,7 @@
       </c>
       <c r="J269" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15579,7 +15579,7 @@
       </c>
       <c r="J270" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15631,7 +15631,7 @@
       </c>
       <c r="J271" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15683,7 +15683,7 @@
       </c>
       <c r="J272" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15735,7 +15735,7 @@
       </c>
       <c r="J273" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15787,7 +15787,7 @@
       </c>
       <c r="J274" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15839,7 +15839,7 @@
       </c>
       <c r="J275" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15891,7 +15891,7 @@
       </c>
       <c r="J276" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15943,7 +15943,7 @@
       </c>
       <c r="J277" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -15996,7 +15996,7 @@
       </c>
       <c r="J278" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16048,7 +16048,7 @@
       </c>
       <c r="J279" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16100,7 +16100,7 @@
       </c>
       <c r="J280" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16153,7 +16153,7 @@
       </c>
       <c r="J281" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16205,7 +16205,7 @@
       </c>
       <c r="J282" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16257,7 +16257,7 @@
       </c>
       <c r="J283" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16309,7 +16309,7 @@
       </c>
       <c r="J284" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16361,7 +16361,7 @@
       </c>
       <c r="J285" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16413,7 +16413,7 @@
       </c>
       <c r="J286" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16465,7 +16465,7 @@
       </c>
       <c r="J287" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16517,7 +16517,7 @@
       </c>
       <c r="J288" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16569,7 +16569,7 @@
       </c>
       <c r="J289" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16622,7 +16622,7 @@
       </c>
       <c r="J290" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16675,7 +16675,7 @@
       </c>
       <c r="J291" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16727,7 +16727,7 @@
       </c>
       <c r="J292" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16779,7 +16779,7 @@
       </c>
       <c r="J293" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16831,7 +16831,7 @@
       </c>
       <c r="J294" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16883,7 +16883,7 @@
       </c>
       <c r="J295" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16935,7 +16935,7 @@
       </c>
       <c r="J296" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -16987,7 +16987,7 @@
       </c>
       <c r="J297" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -17039,7 +17039,7 @@
       </c>
       <c r="J298" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -17091,7 +17091,7 @@
       </c>
       <c r="J299" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -17144,7 +17144,7 @@
       </c>
       <c r="J300" s="14" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>
@@ -17196,7 +17196,7 @@
       </c>
       <c r="J301" s="16" t="inlineStr">
         <is>
-          <t>2026-07-23 20:08:50</t>
+          <t>2026-07-24 08:34:59</t>
         </is>
       </c>
     </row>

</xml_diff>